<commit_message>
Verdere bestellinglijst. Aangevuld met Aisler en Kiwi Tech
</commit_message>
<xml_diff>
--- a/documenten/Bestellijst-GSTEM.xlsx
+++ b/documenten/Bestellijst-GSTEM.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet name="Bestellijst" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Legende" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Bestelschema PCB" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bestellijst'!$A$2:$J$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bestellijst'!$A$2:$J$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -55,7 +56,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -79,6 +80,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
@@ -89,7 +95,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E1D5E7"/>
       </patternFill>
     </fill>
   </fills>
@@ -133,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -172,6 +188,15 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -181,6 +206,25 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -546,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -556,7 +600,7 @@
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
     <col width="52" customWidth="1" min="9" max="9"/>
     <col width="52" customWidth="1" min="10" max="10"/>
   </cols>
@@ -564,7 +608,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Bestellijst G-Stem meettoestel - prijzen incl. btw, gezocht op antratek.be (2026-10-06)</t>
+          <t>Bestellijst G-Stem meettoestel - prijzen incl. btw (Kiwi Electronics + antratek + AISLER, 2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -678,7 +722,7 @@
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>1x toestel, 1x LoRa-ontvanger laptop; antenne inbegrepen</t>
+          <t>1x toestel, 1x LoRa-ontvanger laptop; antenne inbegrepen. Kiwi verkoopt XIAO (EUR 8,46) + Wio-SX1262 (EUR 5,43) apart, maar de Wio-module is daar NIET op voorraad</t>
         </is>
       </c>
     </row>
@@ -711,34 +755,38 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>9-DOF Absolute Orientation IMU Fusion Breakout - BNO055</t>
+          <t>Adafruit 9-DOF Orientation IMU Fusion Breakout - BNO085 (BNO080) - STEMMA QT/Qwiic</t>
         </is>
       </c>
       <c r="D6" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>36.24</v>
+        <v>32.05</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>36.24</v>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>antratek</t>
+        <v>32.05</v>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>kiwi</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>antratek.be</t>
+          <t>Kiwi Electronics</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr">
         <is>
-          <t>https://www.antratek.be/9-dof-absolute-orientation-imu-fusion-breakout-bno055</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr"/>
+          <t>https://www.kiwi-electronics.com/nl/adafruit-9-dof-orientation-imu-fusion-breakout-bno085-bno080-stemma-qt-qwiic-11273</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>Goedkoper en nieuwer dan de BNO055 (anratek EUR 36,24)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -753,36 +801,36 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Atmospheric Sensor Breakout - BME280 (Qwiic)</t>
+          <t>Adafruit BMP581 I2C/SPI Druk- en Temperatuursensor - STEMMA QT</t>
         </is>
       </c>
       <c r="D7" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>19.97</v>
+        <v>10.88</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>19.97</v>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>antratek</t>
+        <v>10.88</v>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>kiwi</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>antratek.be</t>
+          <t>Kiwi Electronics</t>
         </is>
       </c>
       <c r="I7" s="10" t="inlineStr">
         <is>
-          <t>https://www.antratek.be/atmospheric-sensor-breakout-bme280</t>
+          <t>https://www.kiwi-electronics.com/nl/adafruit-bmp581-i2c-spi-druk-en-temperatuursensor-stemma-qt-20534</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Goedkoopst/leverbaar alternatief voor BMP390; minder nauwkeurig (EUR 1 hPa i.p.v. 0,03 hPa)</t>
+          <t>Nauwkeuriger dan BME280; BMP390L is bij Kiwi uit voorraad en niet op antratek</t>
         </is>
       </c>
     </row>
@@ -807,7 +855,7 @@
       </c>
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
-      <c r="G8" s="11" t="inlineStr">
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>geen link</t>
         </is>
@@ -820,7 +868,7 @@
       <c r="I8" s="6" t="inlineStr"/>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Niet op antratek.be. Alternatief: LG290P RTK (EUR 217,74) of ZED-F9P (EUR 302,44)</t>
+          <t>Niet bij Kiwi (alleen niet-RTK L76K) of antratek. Alternatief: LG290P RTK (EUR 217,74) of ZED-F9P (EUR 302,44)</t>
         </is>
       </c>
     </row>
@@ -853,36 +901,36 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>GPS/GNSS Magnetic Mount Antenna SMA - 3m, SparkFun GPS-14986</t>
+          <t>GPS Antenne - Externe Actieve Antenne - 3-5V 28dB 5 Meter SMA</t>
         </is>
       </c>
       <c r="D10" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>19.3</v>
+        <v>16.93</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>antratek</t>
+        <v>16.93</v>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>kiwi</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>antratek.be</t>
+          <t>Kiwi Electronics</t>
         </is>
       </c>
       <c r="I10" s="10" t="inlineStr">
         <is>
-          <t>https://www.antratek.be/gps-gnss-magnetic-mount-antenna-sma-3m</t>
+          <t>https://www.kiwi-electronics.com/nl/gps-antenne-externe-actieve-antenne-3-5v-28db-5-meter-sma-620</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>Goedkoopste passende antenne (L1, multi-constellatie). Upgrade voor dual-band RTK: L1/L5-antenne EUR 120,94</t>
+          <t>Goedkoopste passende actieve SMA-antenne (L1). Upgrade voor dual-band RTK: L1/L5-antenne EUR 120,94</t>
         </is>
       </c>
     </row>
@@ -928,7 +976,7 @@
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>Bulkhead-bevestiging apart controleren</t>
+          <t>Goedkoper op antratek (EUR 3,57) dan Kiwi (EUR 4,22); bulkhead-bevestiging apart controleren</t>
         </is>
       </c>
     </row>
@@ -953,7 +1001,7 @@
       </c>
       <c r="E12" s="5" t="n"/>
       <c r="F12" s="5" t="n"/>
-      <c r="G12" s="12" t="inlineStr">
+      <c r="G12" s="13" t="inlineStr">
         <is>
           <t>al in bezit</t>
         </is>
@@ -1003,7 +1051,7 @@
       </c>
       <c r="E14" s="5" t="n"/>
       <c r="F14" s="5" t="n"/>
-      <c r="G14" s="12" t="inlineStr">
+      <c r="G14" s="13" t="inlineStr">
         <is>
           <t>al in bezit</t>
         </is>
@@ -1037,7 +1085,7 @@
       </c>
       <c r="E15" s="5" t="n"/>
       <c r="F15" s="5" t="n"/>
-      <c r="G15" s="12" t="inlineStr">
+      <c r="G15" s="13" t="inlineStr">
         <is>
           <t>al in bezit</t>
         </is>
@@ -1075,7 +1123,7 @@
       </c>
       <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="n"/>
-      <c r="G16" s="12" t="inlineStr">
+      <c r="G16" s="13" t="inlineStr">
         <is>
           <t>al in bezit</t>
         </is>
@@ -1111,22 +1159,26 @@
       <c r="D17" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="11" t="inlineStr">
-        <is>
-          <t>geen link</t>
+      <c r="E17" s="8" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>schatting</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>componentenwinkel</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>Niet op antratek.be</t>
+          <t>Niet bij Kiwi of antratek; prijs is een schatting (Mouser/LCSC)</t>
         </is>
       </c>
     </row>
@@ -1149,22 +1201,26 @@
       <c r="D18" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="11" t="inlineStr">
-        <is>
-          <t>geen link</t>
+      <c r="E18" s="8" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>schatting</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>componentenwinkel</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr"/>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>Niet op antratek.be</t>
+          <t>Niet bij Kiwi of antratek; prijs is een schatting</t>
         </is>
       </c>
     </row>
@@ -1187,7 +1243,7 @@
       <c r="D19" s="5" t="n"/>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
-      <c r="G19" s="13" t="inlineStr">
+      <c r="G19" s="15" t="inlineStr">
         <is>
           <t>niet nodig</t>
         </is>
@@ -1203,7 +1259,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Print en verbindingen</t>
+          <t>Draagprint (PCB bij AISLER)</t>
         </is>
       </c>
       <c r="B20" s="4" t="n"/>
@@ -1219,86 +1275,64 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
+          <t>Draagprint (PCB bij AISLER)</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Draagprint (printplaat)</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>2-laags 1,6 mm HASL, set van 3 stuks - AISLER</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>10.92</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>32.76</v>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>aisler</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>AISLER</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="inlineStr">
+        <is>
+          <t>https://aisler.net</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>Schatting 75 cm2 (100x75 mm), incl. btw; Budget-service. Formule: EUR 12,00 + EUR 0,067/cm2 x oppervlak x aantal. AISLER levert in sets van 3; gratis verzending. Definitieve maat volgt uit de KiCad-layout</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
           <t>Print en verbindingen</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>Level shifter 3,3 V &lt;-&gt; 5 V</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>Logic Level Converter Bi-Directional (alternatief voor TXB0104)</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="8" t="n">
-        <v>4.78</v>
-      </c>
-      <c r="F21" s="8" t="n">
-        <v>4.78</v>
-      </c>
-      <c r="G21" s="9" t="inlineStr">
-        <is>
-          <t>antratek</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>antratek.be</t>
-        </is>
-      </c>
-      <c r="I21" s="10" t="inlineStr">
-        <is>
-          <t>https://www.antratek.be/logic-level-converter-bi-directional-bob-12009</t>
-        </is>
-      </c>
-      <c r="J21" s="6" t="inlineStr">
-        <is>
-          <t>Gekozen TXB0104 niet op antratek; dit is een bruikbaar alternatief</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Print en verbindingen</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>Schroefklem 4-pins 3,5 mm</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>KF128/KF301</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="5" t="n"/>
-      <c r="G22" s="11" t="inlineStr">
-        <is>
-          <t>geen link</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I22" s="6" t="inlineStr"/>
-      <c r="J22" s="6" t="inlineStr">
-        <is>
-          <t>Niet op antratek.be; antratek heeft wel terminal-block pluggen</t>
-        </is>
-      </c>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
+      <c r="I22" s="4" t="n"/>
+      <c r="J22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1308,33 +1342,41 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Sockets</t>
+          <t>Level shifter 3,3 V &lt;-&gt; 5 V</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Dual-wipe (ESP32) + precisie voor de rest</t>
+          <t>8-kanaals bidirectionele Logic Level Converter - TXB0108</t>
         </is>
       </c>
       <c r="D23" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="n"/>
+      <c r="E23" s="8" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>8.699999999999999</v>
+      </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
-          <t>geen link</t>
+          <t>kiwi</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I23" s="6" t="inlineStr"/>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="inlineStr">
+        <is>
+          <t>https://www.kiwi-electronics.com/nl/8-channel-bi-directional-logic-level-converter-txb0108-836</t>
+        </is>
+      </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>Niet op antratek.be</t>
+          <t>Past bij de gekozen TXB-serie; antratek-alternatief BSS138-converter EUR 4,78</t>
         </is>
       </c>
     </row>
@@ -1346,33 +1388,37 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Power-LED + serieweerstand</t>
+          <t>Schroefklem 4-pins 3,5 mm</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Status voeding</t>
+          <t>KF128/KF301</t>
         </is>
       </c>
       <c r="D24" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="n"/>
-      <c r="G24" s="11" t="inlineStr">
-        <is>
-          <t>geen link</t>
+      <c r="E24" s="8" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G24" s="14" t="inlineStr">
+        <is>
+          <t>schatting</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>componentenwinkel</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr"/>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>Niet op antratek.be</t>
+          <t>Niet bij Kiwi (alleen 3-weg) of antratek; prijs schatting</t>
         </is>
       </c>
     </row>
@@ -1384,33 +1430,37 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Ontkoppelcondensatoren</t>
+          <t>Sockets</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>100 nF + 10 uF per modulevoedingspin</t>
+          <t>Dual-wipe (ESP32) + precisie voor de rest</t>
         </is>
       </c>
       <c r="D25" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="5" t="n"/>
-      <c r="F25" s="5" t="n"/>
-      <c r="G25" s="11" t="inlineStr">
-        <is>
-          <t>geen link</t>
+      <c r="E25" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="G25" s="14" t="inlineStr">
+        <is>
+          <t>schatting</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>componentenwinkel</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>Niet op antratek.be</t>
+          <t>Niet bij Kiwi of antratek; prijs schatting (zie pcb-methodes-kosten)</t>
         </is>
       </c>
     </row>
@@ -1422,33 +1472,41 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Bulk-elco</t>
+          <t>Power-LED + serieweerstand</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>100 uF / 16 V op de 5 V-ingang</t>
+          <t>3 mm LED rood (10-pack) + weerstand 330 Ohm (10-pack)</t>
         </is>
       </c>
       <c r="D26" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26" s="5" t="n"/>
+      <c r="E26" s="8" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="F26" s="8" t="n">
+        <v>2.16</v>
+      </c>
       <c r="G26" s="11" t="inlineStr">
         <is>
-          <t>geen link</t>
+          <t>kiwi</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I26" s="6" t="inlineStr"/>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t>https://www.kiwi-electronics.com/nl/3mm-led-diffuus-rood-10-pack-3085</t>
+        </is>
+      </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>Niet op antratek.be</t>
+          <t>10-packs: 1 LED + 1 weerstand nodig; weerstand EUR 0,96; rest overschot</t>
         </is>
       </c>
     </row>
@@ -1460,33 +1518,41 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>I2C-pull-ups op de print</t>
+          <t>Ontkoppelcondensatoren</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Niet nodig; breakouts hebben ze al</t>
+          <t>Keramische condensator kit (15 soorten, 450 st.) - dekt 100 nF + 10 uF</t>
         </is>
       </c>
       <c r="D27" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E27" s="5" t="n"/>
-      <c r="F27" s="5" t="n"/>
-      <c r="G27" s="13" t="inlineStr">
-        <is>
-          <t>niet nodig</t>
+        <v>1</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>10.27</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>10.27</v>
+      </c>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>kiwi</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I27" s="6" t="inlineStr"/>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="I27" s="10" t="inlineStr">
+        <is>
+          <t>https://www.kiwi-electronics.com/nl/keramische-condensator-kit-in-doos-15-soorten-450-stuks-10492</t>
+        </is>
+      </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>2 reserve-footprints</t>
+          <t>Kit i.p.v. losse condensatoren</t>
         </is>
       </c>
     </row>
@@ -1498,119 +1564,135 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Montage</t>
+          <t>Bulk-elco</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>M3-schroeven, moeren, standoffs, nylon spacers</t>
+          <t>100 uF / 16 V op de 5 V-ingang</t>
         </is>
       </c>
       <c r="D28" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
+      <c r="E28" s="8" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F28" s="8" t="n">
+        <v>0.59</v>
+      </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>geen link</t>
+          <t>kiwi</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="I28" s="10" t="inlineStr">
+        <is>
+          <t>https://www.kiwi-electronics.com/nl/100uf-16v-condensator-440</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Print en verbindingen</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>I2C-pull-ups op de print</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Niet nodig; breakouts hebben ze al</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="15" t="inlineStr">
+        <is>
+          <t>niet nodig</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I28" s="6" t="inlineStr"/>
-      <c r="J28" s="6" t="inlineStr">
-        <is>
-          <t>Niet op antratek.be</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>Kabels en verbruik (in bezit)</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="n"/>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="n"/>
-      <c r="G29" s="4" t="n"/>
-      <c r="H29" s="4" t="n"/>
-      <c r="I29" s="4" t="n"/>
-      <c r="J29" s="4" t="n"/>
+      <c r="I29" s="6" t="inlineStr"/>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>2 reserve-footprints</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Kabels en verbruik (in bezit)</t>
+          <t>Print en verbindingen</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>USB-C datakabel</t>
+          <t>Montage</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Eigen kabel</t>
+          <t>M3-schroeven, moeren, standoffs, nylon spacers</t>
         </is>
       </c>
       <c r="D30" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E30" s="5" t="n"/>
-      <c r="F30" s="5" t="n"/>
-      <c r="G30" s="12" t="inlineStr">
-        <is>
-          <t>al in bezit</t>
+      <c r="E30" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F30" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>schatting</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>componentenwinkel</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr"/>
-      <c r="J30" s="6" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>Niet bij Kiwi of antratek; prijs schatting</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Kabels en verbruik (in bezit)</t>
         </is>
       </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>Dupont-/siliconendraad</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>Heeft de gebruiker</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="12" t="inlineStr">
-        <is>
-          <t>al in bezit</t>
-        </is>
-      </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I31" s="6" t="inlineStr"/>
-      <c r="J31" s="6" t="inlineStr"/>
+      <c r="B31" s="4" t="n"/>
+      <c r="C31" s="4" t="n"/>
+      <c r="D31" s="4" t="n"/>
+      <c r="E31" s="4" t="n"/>
+      <c r="F31" s="4" t="n"/>
+      <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="n"/>
+      <c r="I31" s="4" t="n"/>
+      <c r="J31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -1620,12 +1702,12 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>USB A-kabel LoRa-ontvanger</t>
+          <t>USB-C datakabel</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>USB-A naar USB-C voor de XIAO (heeft de gebruiker)</t>
+          <t>Eigen kabel</t>
         </is>
       </c>
       <c r="D32" s="7" t="n">
@@ -1633,7 +1715,7 @@
       </c>
       <c r="E32" s="5" t="n"/>
       <c r="F32" s="5" t="n"/>
-      <c r="G32" s="12" t="inlineStr">
+      <c r="G32" s="13" t="inlineStr">
         <is>
           <t>al in bezit</t>
         </is>
@@ -1654,12 +1736,12 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Gereedschap</t>
+          <t>Dupont-/siliconendraad</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Schuifmaat, soldeerbout, tin, flux, multimeter, USB-serieel adapter</t>
+          <t>Heeft de gebruiker</t>
         </is>
       </c>
       <c r="D33" s="7" t="n">
@@ -1667,7 +1749,7 @@
       </c>
       <c r="E33" s="5" t="n"/>
       <c r="F33" s="5" t="n"/>
-      <c r="G33" s="12" t="inlineStr">
+      <c r="G33" s="13" t="inlineStr">
         <is>
           <t>al in bezit</t>
         </is>
@@ -1680,36 +1762,54 @@
       <c r="I33" s="6" t="inlineStr"/>
       <c r="J33" s="6" t="inlineStr"/>
     </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>Mock-up (vliegtuigje)</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="n"/>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4" t="n"/>
-      <c r="E34" s="4" t="n"/>
-      <c r="F34" s="4" t="n"/>
-      <c r="G34" s="4" t="n"/>
-      <c r="H34" s="4" t="n"/>
-      <c r="I34" s="4" t="n"/>
-      <c r="J34" s="4" t="n"/>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Kabels en verbruik (in bezit)</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>USB A-kabel LoRa-ontvanger</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>USB-A naar USB-C voor de XIAO (heeft de gebruiker)</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="5" t="n"/>
+      <c r="F34" s="5" t="n"/>
+      <c r="G34" s="13" t="inlineStr">
+        <is>
+          <t>al in bezit</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr"/>
+      <c r="J34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Mock-up (vliegtuigje)</t>
+          <t>Kabels en verbruik (in bezit)</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Arduino</t>
+          <t>Gereedschap</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Arduino Uno (heeft de gebruiker thuis)</t>
+          <t>Schuifmaat, soldeerbout, tin, flux, multimeter, USB-serieel adapter</t>
         </is>
       </c>
       <c r="D35" s="7" t="n">
@@ -1717,7 +1817,7 @@
       </c>
       <c r="E35" s="5" t="n"/>
       <c r="F35" s="5" t="n"/>
-      <c r="G35" s="12" t="inlineStr">
+      <c r="G35" s="13" t="inlineStr">
         <is>
           <t>al in bezit</t>
         </is>
@@ -1728,45 +1828,23 @@
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr"/>
-      <c r="J35" s="6" t="inlineStr">
-        <is>
-          <t>Referentie antratek: Arduino Uno Rev3 (EUR 41,75)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="J35" s="6" t="inlineStr"/>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>Mock-up (vliegtuigje)</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>Servo's</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>Bestaande voorraad (&gt; 3)</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E36" s="5" t="n"/>
-      <c r="F36" s="5" t="n"/>
-      <c r="G36" s="12" t="inlineStr">
-        <is>
-          <t>al in bezit</t>
-        </is>
-      </c>
-      <c r="H36" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I36" s="6" t="inlineStr"/>
-      <c r="J36" s="6" t="inlineStr"/>
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="4" t="n"/>
+      <c r="D36" s="4" t="n"/>
+      <c r="E36" s="4" t="n"/>
+      <c r="F36" s="4" t="n"/>
+      <c r="G36" s="4" t="n"/>
+      <c r="H36" s="4" t="n"/>
+      <c r="I36" s="4" t="n"/>
+      <c r="J36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -1776,12 +1854,12 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Servo-voeding</t>
+          <t>Arduino</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Aparte buck-converter</t>
+          <t>Arduino Uno (heeft de gebruiker thuis)</t>
         </is>
       </c>
       <c r="D37" s="7" t="n">
@@ -1789,7 +1867,7 @@
       </c>
       <c r="E37" s="5" t="n"/>
       <c r="F37" s="5" t="n"/>
-      <c r="G37" s="12" t="inlineStr">
+      <c r="G37" s="13" t="inlineStr">
         <is>
           <t>al in bezit</t>
         </is>
@@ -1800,7 +1878,11 @@
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr"/>
-      <c r="J37" s="6" t="inlineStr"/>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>Referentie antratek: Arduino Uno Rev3 (EUR 41,75)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -1810,20 +1892,20 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Romp en roeren</t>
+          <t>Servo's</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Eigen 3D-print</t>
+          <t>Bestaande voorraad (&gt; 3)</t>
         </is>
       </c>
       <c r="D38" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E38" s="5" t="n"/>
       <c r="F38" s="5" t="n"/>
-      <c r="G38" s="12" t="inlineStr">
+      <c r="G38" s="13" t="inlineStr">
         <is>
           <t>al in bezit</t>
         </is>
@@ -1837,42 +1919,211 @@
       <c r="J38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="14" t="inlineStr">
-        <is>
-          <t>Totaal te bestellen bij antratek (excl. geen-link-onderdelen)</t>
-        </is>
-      </c>
-      <c r="B39" s="15" t="n"/>
-      <c r="C39" s="15" t="n"/>
-      <c r="D39" s="15" t="n"/>
-      <c r="E39" s="15" t="n"/>
-      <c r="F39" s="16">
-        <f>SUMIF(G3:G38,"antratek",F3:F38)</f>
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Mock-up (vliegtuigje)</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Servo-voeding</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Aparte buck-converter</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="13" t="inlineStr">
+        <is>
+          <t>al in bezit</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr"/>
+      <c r="J39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Mock-up (vliegtuigje)</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>Romp en roeren</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Eigen 3D-print</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="5" t="n"/>
+      <c r="F40" s="5" t="n"/>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>al in bezit</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I40" s="6" t="inlineStr"/>
+      <c r="J40" s="6" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>Totaal te bestellen bij Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="B42" s="18" t="n"/>
+      <c r="C42" s="18" t="n"/>
+      <c r="D42" s="18" t="n"/>
+      <c r="E42" s="18" t="n"/>
+      <c r="F42" s="19">
+        <f>SUMIF(G3:G40,"kiwi",F3:F40)</f>
         <v/>
       </c>
-      <c r="G39" s="15" t="n"/>
-      <c r="H39" s="15" t="n"/>
-      <c r="I39" s="15" t="n"/>
-      <c r="J39" s="15" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="17" t="inlineStr">
-        <is>
-          <t>Let op: prijzen onder voorbehoud (anratek 2026-10-06). Niet-gevonden onderdelen staan op 'geen link' en zijn niet in het totaal opgenomen.</t>
+      <c r="G42" s="18" t="n"/>
+      <c r="H42" s="18" t="n"/>
+      <c r="I42" s="18" t="n"/>
+      <c r="J42" s="18" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>Totaal te bestellen bij antratek</t>
+        </is>
+      </c>
+      <c r="B43" s="18" t="n"/>
+      <c r="C43" s="18" t="n"/>
+      <c r="D43" s="18" t="n"/>
+      <c r="E43" s="18" t="n"/>
+      <c r="F43" s="19">
+        <f>SUMIF(G3:G40,"antratek",F3:F40)</f>
+        <v/>
+      </c>
+      <c r="G43" s="18" t="n"/>
+      <c r="H43" s="18" t="n"/>
+      <c r="I43" s="18" t="n"/>
+      <c r="J43" s="18" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>Subtotaal onderdelen (Kiwi + antratek)</t>
+        </is>
+      </c>
+      <c r="B44" s="18" t="n"/>
+      <c r="C44" s="18" t="n"/>
+      <c r="D44" s="18" t="n"/>
+      <c r="E44" s="18" t="n"/>
+      <c r="F44" s="19">
+        <f>F42+F43</f>
+        <v/>
+      </c>
+      <c r="G44" s="18" t="n"/>
+      <c r="H44" s="18" t="n"/>
+      <c r="I44" s="18" t="n"/>
+      <c r="J44" s="18" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="inlineStr">
+        <is>
+          <t>Totaal draagprint bij AISLER (3 stuks)</t>
+        </is>
+      </c>
+      <c r="B45" s="18" t="n"/>
+      <c r="C45" s="18" t="n"/>
+      <c r="D45" s="18" t="n"/>
+      <c r="E45" s="18" t="n"/>
+      <c r="F45" s="19">
+        <f>SUMIF(G3:G40,"aisler",F3:F40)</f>
+        <v/>
+      </c>
+      <c r="G45" s="18" t="n"/>
+      <c r="H45" s="18" t="n"/>
+      <c r="I45" s="18" t="n"/>
+      <c r="J45" s="18" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>Totaal PCB-onderdelen (schatting, apart bestellen)</t>
+        </is>
+      </c>
+      <c r="B46" s="18" t="n"/>
+      <c r="C46" s="18" t="n"/>
+      <c r="D46" s="18" t="n"/>
+      <c r="E46" s="18" t="n"/>
+      <c r="F46" s="19">
+        <f>SUMIF(G3:G40,"schatting",F3:F40)</f>
+        <v/>
+      </c>
+      <c r="G46" s="18" t="n"/>
+      <c r="H46" s="18" t="n"/>
+      <c r="I46" s="18" t="n"/>
+      <c r="J46" s="18" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>Totaal alles (incl. print + PCB-onderdelen)</t>
+        </is>
+      </c>
+      <c r="B47" s="18" t="n"/>
+      <c r="C47" s="18" t="n"/>
+      <c r="D47" s="18" t="n"/>
+      <c r="E47" s="18" t="n"/>
+      <c r="F47" s="19">
+        <f>F44+F45+F46</f>
+        <v/>
+      </c>
+      <c r="G47" s="18" t="n"/>
+      <c r="H47" s="18" t="n"/>
+      <c r="I47" s="18" t="n"/>
+      <c r="J47" s="18" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="20" t="inlineStr">
+        <is>
+          <t>Let op: prijzen onder voorbehoud (Kiwi Electronics + antratek + AISLER, 2026-10-06). De PCB-onderdelen op status 'schatting' zijn benaderd (o.a. sockets, discrete voeding, LDO, schroefklem, M3-montage). Het 'geen link'-onderdeel (RTK-module LC29H) is niet in de totalen opgenomen. Details: GEBRUIKER/data/bestelschema-pcb.md.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J38"/>
-  <mergeCells count="9">
-    <mergeCell ref="A39:E39"/>
+  <autoFilter ref="A2:J40"/>
+  <mergeCells count="15">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A36:J36"/>
+    <mergeCell ref="A31:J31"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A22:J22"/>
     <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A42:E42"/>
     <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A34:J34"/>
-    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A46:E46"/>
     <mergeCell ref="A20:J20"/>
+    <mergeCell ref="A44:E44"/>
     <mergeCell ref="A13:J13"/>
   </mergeCells>
   <hyperlinks>
@@ -1882,6 +2133,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1893,68 +2148,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="B1" s="18" t="inlineStr">
+      <c r="B1" s="21" t="inlineStr">
         <is>
           <t>Betekenis</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>kiwi</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Aankooplink gevonden op Kiwi Electronics (kiwi-electronics.com)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>antratek</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Aankooplink gevonden op antratek.be</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Aankooplink gevonden op antratek.be (goedkoper of als reserve)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>aisler</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Gefabriceerd bij AISLER (EU); print zelf, geen componenten</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>schatting</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Prijs is een schatting; apart te bestellen bij een componentenwinkel</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>al in bezit</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Heeft de gebruiker al; niet aankopen</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t>geen link</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Niet gevonden op antratek.be; niet elders gezocht</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Niet gevonden bij Kiwi of antratek; nog geen prijs</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>niet nodig</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Bewust niet voorzien</t>
         </is>
@@ -1963,4 +2254,480 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="29" t="inlineStr">
+        <is>
+          <t>Bestelschema draagprint bij AISLER - schatting (2026-10-06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>AISLER-productie - 2-laags 1,6 mm HASL Budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Formule: EUR 12,00 job fee + EUR 0,067/cm2 x oppervlak x aantal (sets van 3, gratis verzending, productie vanaf 2 werkdagen)</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>Oppervlak</t>
+        </is>
+      </c>
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>3 stuks incl. btw</t>
+        </is>
+      </c>
+      <c r="C4" s="31" t="inlineStr">
+        <is>
+          <t>6 stuks incl. btw</t>
+        </is>
+      </c>
+      <c r="D4" s="31" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>60 cm2 (bv. 100x60)</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>29.11</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>43.71</v>
+      </c>
+      <c r="D5" s="6" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>75 cm2 (100x75, aanname)</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>32.76</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>50.99</v>
+      </c>
+      <c r="D6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>90 cm2 (120x75)</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>36.41</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="D7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>100 cm2 (100x100)</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>38.84</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>63.16</v>
+      </c>
+      <c r="D8" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="30" t="inlineStr">
+        <is>
+          <t>Onderdelen op de print</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>Onderdeel</t>
+        </is>
+      </c>
+      <c r="B11" s="31" t="inlineStr">
+        <is>
+          <t>Prijs (EUR)</t>
+        </is>
+      </c>
+      <c r="C11" s="31" t="inlineStr">
+        <is>
+          <t>Leverancier</t>
+        </is>
+      </c>
+      <c r="D11" s="31" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Sockets (dual-wipe + precisie)</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>componentenwinkel (schatting)</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Voedingsbescherming (2 A PTC + DMG2301L + SMBJ10A)</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>componentenwinkel (schatting)</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>LDO AP2112K-3.3</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>componentenwinkel (schatting)</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Schroefklem 4-pins 3,5 mm (KF128/KF301)</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>componentenwinkel (schatting)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>M3-schroeven, moeren, standoffs, spacers</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>componentenwinkel (schatting)</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="31" t="inlineStr">
+        <is>
+          <t>Subtotaal apart te bestellen</t>
+        </is>
+      </c>
+      <c r="B17" s="32" t="n">
+        <v>10.85</v>
+      </c>
+      <c r="C17" s="31" t="inlineStr">
+        <is>
+          <t>schatting</t>
+        </is>
+      </c>
+      <c r="D17" s="31" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>TXB0108 level shifter</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>LED + serieweerstand (per bord gebruikt)</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Ontkoppelcondensatoren (per bord gebruikt)</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Bulk-elco 100 uF</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="31" t="inlineStr">
+        <is>
+          <t>Subtotaal al in hoofd-bestellijst</t>
+        </is>
+      </c>
+      <c r="B22" s="32" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="C22" s="31" t="inlineStr">
+        <is>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="D22" s="31" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="31" t="inlineStr">
+        <is>
+          <t>Totaal onderdelen op de print (met TXB0108)</t>
+        </is>
+      </c>
+      <c r="B23" s="32" t="n">
+        <v>20.86</v>
+      </c>
+      <c r="C23" s="31" t="inlineStr">
+        <is>
+          <t>met TXB0104-IC direct: ca. 13,96</t>
+        </is>
+      </c>
+      <c r="D23" s="31" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>Totalen (3 borden, incl. btw)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>AISLER print, 3 stuks, 75 cm2 Budget</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="n">
+        <v>32.76</v>
+      </c>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>Onderdelen op de print</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="n">
+        <v>20.86</v>
+      </c>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="31" t="inlineStr">
+        <is>
+          <t>Totaal</t>
+        </is>
+      </c>
+      <c r="B28" s="32" t="n">
+        <v>53.62</v>
+      </c>
+      <c r="C28" s="31" t="n"/>
+      <c r="D28" s="31" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Waarvan al in de hoofd-bestellijst</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="C29" s="6" t="n"/>
+      <c r="D29" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="31" t="inlineStr">
+        <is>
+          <t>Werkelijk nieuw te bestellen</t>
+        </is>
+      </c>
+      <c r="B30" s="32" t="n">
+        <v>43.61</v>
+      </c>
+      <c r="C30" s="31" t="n"/>
+      <c r="D30" s="31" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>Bestelvolgorde</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>1. PCB ontwerpen in KiCad; layout afronden, DRC, Gerbers/ODB++ exporteren</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="n"/>
+      <c r="C33" s="6" t="n"/>
+      <c r="D33" s="6" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>2. Bordafmeting definitief nameten en AISLER-calculator controleren</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n"/>
+      <c r="C34" s="6" t="n"/>
+      <c r="D34" s="6" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>3. Print bestellen bij AISLER (3 of 6 stuks, Budget-service)</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n"/>
+      <c r="C35" s="6" t="n"/>
+      <c r="D35" s="6" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>4. Tegelijk de 'schatting'-onderdelen bestellen (sockets, voeding, LDO, klem, montage)</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n"/>
+      <c r="C36" s="6" t="n"/>
+      <c r="D36" s="6" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>5. Kiwi/antratek-bestelling: level shifter, LED, condensatoren, bulk-elco</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="n"/>
+      <c r="C37" s="6" t="n"/>
+      <c r="D37" s="6" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>6. Rendering vergelijken met het echte bord, daarna solderen</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="n"/>
+      <c r="C38" s="6" t="n"/>
+      <c r="D38" s="6" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A10:D10"/>
+    <mergeCell ref="A32:D32"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Bestellingen, models, daw.io schema
</commit_message>
<xml_diff>
--- a/documenten/Bestellijst-GSTEM.xlsx
+++ b/documenten/Bestellijst-GSTEM.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Bestellijst" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Legende" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Bestelschema PCB" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bestellijst" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legende" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bestelschema PCB" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bestelbaarheid" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bestellijst'!$A$2:$J$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bestellijst'!$A$2:$J$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -56,7 +57,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -85,7 +86,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -95,7 +96,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -105,7 +106,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E1D5E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -149,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -197,6 +213,12 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -208,11 +230,14 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -590,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -608,7 +633,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Bestellijst G-Stem meettoestel - prijzen incl. btw (Kiwi Electronics + antratek + AISLER, 2026-10-06)</t>
+          <t>Bestellijst G-Stem meettoestel - prijzen incl. btw (Kiwi + antratek + Eckstein + TME + Mouser + HESTORE + TinyTronics + AISLER, 2026-10-06)</t>
         </is>
       </c>
     </row>
@@ -842,33 +867,41 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>RTK-GNSS-module</t>
+          <t>RTK-GNSS-module (breakout)</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Quectel LC29H(DA)</t>
+          <t>Waveshare LC29H(DA) GPS/RTK HAT (SKU 25279), incl. actieve dual-band L1/L5-antenne + IPEX-naar-SMA-kabel + 40-pins header</t>
         </is>
       </c>
       <c r="D8" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
+      <c r="E8" s="8" t="n">
+        <v>71.39</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>71.39</v>
+      </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
-          <t>geen link</t>
+          <t>eckstein</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr"/>
+          <t>Eckstein (Duitsland, EU)</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>https://eckstein-shop.de/lc29h-dual-band-gps-module-raspberry-pi_1</t>
+        </is>
+      </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Niet bij Kiwi (alleen niet-RTK L76K) of antratek. Alternatief: LG290P RTK (EUR 217,74) of ZED-F9P (EUR 302,44)</t>
+          <t>GEKOZEN door gebruiker (2026-10-06): Eckstein, art. WS25279 / EAN 4060137304156, EUR 71,39 incl. Kant-en-klare breakout/HAT (geen losse SMD-module), 65x30,5 mm. Alternatieven: Kamami (PL) ca. EUR 63; Botland (PL/DE) EUR 70,50; HESTORE (HU) EUR 91,21 excl. (ca. EUR 110 incl.). Niet-EU: 7Semi LC29HDA RTK Board (Qwiic/USB-C, ca. USD 42, India)</t>
         </is>
       </c>
     </row>
@@ -896,41 +929,33 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>GNSS-antenne (actief, SMA)</t>
+          <t>GNSS-antenne (actief, L1/L5, SMA)</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>GPS Antenne - Externe Actieve Antenne - 3-5V 28dB 5 Meter SMA</t>
+          <t>Inbegrepen bij de Waveshare LC29H(DA) HAT (dual-band actieve antenne)</t>
         </is>
       </c>
       <c r="D10" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="8" t="n">
-        <v>16.93</v>
-      </c>
-      <c r="F10" s="8" t="n">
-        <v>16.93</v>
-      </c>
-      <c r="G10" s="11" t="inlineStr">
-        <is>
-          <t>kiwi</t>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>al in bezit</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Kiwi Electronics</t>
-        </is>
-      </c>
-      <c r="I10" s="10" t="inlineStr">
-        <is>
-          <t>https://www.kiwi-electronics.com/nl/gps-antenne-externe-actieve-antenne-3-5v-28db-5-meter-sma-620</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr"/>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>Goedkoopste passende actieve SMA-antenne (L1). Upgrade voor dual-band RTK: L1/L5-antenne EUR 120,94</t>
+          <t>Aparte antenne vervalt: de HAT levert een betere dual-band L1/L5-antenne mee (bespaart EUR 16,93 t.o.v. de losse Kiwi L1-antenne)</t>
         </is>
       </c>
     </row>
@@ -1153,32 +1178,36 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>2 A PTC + P-MOSFET DMG2301L + TVS SMBJ10A</t>
+          <t>2 A PTC Littelfuse 1812L200/16 + TVS SMBJ10A-TR (zonder P-MOSFET)</t>
         </is>
       </c>
       <c r="D17" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
-          <t>schatting</t>
+          <t>mouser</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>componentenwinkel</t>
-        </is>
-      </c>
-      <c r="I17" s="6" t="inlineStr"/>
+          <t>Mouser.be / DigiKey (EU-magazijn)</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/ProductDetail/Littelfuse/1812L200-16DR</t>
+        </is>
+      </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>Niet bij Kiwi of antratek; prijs is een schatting (Mouser/LCSC)</t>
+          <t>PTC bij Mouser/DigiKey (EU); TVS SMBJ10A bij TME. P-MOSFET vervalt (beslissing 2026-10-06).</t>
         </is>
       </c>
     </row>
@@ -1190,37 +1219,33 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>LDO 3,3 V</t>
+          <t>Ompoolbeveiliging (P-MOSFET)</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>AP2112K-3.3 (of AMS1117-3.3)</t>
+          <t>P-MOSFET DMG2301L / AO3401A (SOT-23)</t>
         </is>
       </c>
       <c r="D18" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="8" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="F18" s="8" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="G18" s="14" t="inlineStr">
-        <is>
-          <t>schatting</t>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>niet nodig</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>componentenwinkel</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr"/>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>Niet bij Kiwi of antratek; prijs is een schatting</t>
+          <t>BESLISSING 2026-10-06: NIET voorzien. Geen P-MOSFET-ompoolbeveiliging; voorkom omgekeerd aansluiten met een gepolariseerde connector (XT60/JST-XH). Zie data/afgevoerd.md.</t>
         </is>
       </c>
     </row>
@@ -1232,153 +1257,153 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
+          <t>LDO 3,3 V</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>AP2112K-3.3TRG1 (Diodes Inc., SOT-23-5)</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="8" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G19" s="16" t="inlineStr">
+        <is>
+          <t>tme</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>TME (Polen, EU)</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>https://www.tme.eu/en/details/ap2112k-3.3trg1/ldo-fixed-voltage-regulators/diodes-incorporated/</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>8000+ op voorraad bij TME</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Voeding</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
           <t>Aan/uit-schakelaar</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Geen; toestel start bij voeding</t>
         </is>
       </c>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="15" t="inlineStr">
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="15" t="inlineStr">
         <is>
           <t>niet nodig</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr"/>
-      <c r="J19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="I20" s="6" t="inlineStr"/>
+      <c r="J20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Draagprint (PCB bij AISLER)</t>
         </is>
       </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
-      <c r="H20" s="4" t="n"/>
-      <c r="I20" s="4" t="n"/>
-      <c r="J20" s="4" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="n"/>
+      <c r="I21" s="4" t="n"/>
+      <c r="J21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Draagprint (PCB bij AISLER)</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Draagprint (printplaat)</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>2-laags 1,6 mm HASL, set van 3 stuks - AISLER</t>
         </is>
       </c>
-      <c r="D21" s="7" t="n">
+      <c r="D22" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="E21" s="8" t="n">
+      <c r="E22" s="8" t="n">
         <v>10.92</v>
       </c>
-      <c r="F21" s="8" t="n">
+      <c r="F22" s="8" t="n">
         <v>32.76</v>
       </c>
-      <c r="G21" s="16" t="inlineStr">
+      <c r="G22" s="17" t="inlineStr">
         <is>
           <t>aisler</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>AISLER</t>
         </is>
       </c>
-      <c r="I21" s="10" t="inlineStr">
+      <c r="I22" s="10" t="inlineStr">
         <is>
           <t>https://aisler.net</t>
         </is>
       </c>
-      <c r="J21" s="6" t="inlineStr">
+      <c r="J22" s="6" t="inlineStr">
         <is>
           <t>Schatting 75 cm2 (100x75 mm), incl. btw; Budget-service. Formule: EUR 12,00 + EUR 0,067/cm2 x oppervlak x aantal. AISLER levert in sets van 3; gratis verzending. Definitieve maat volgt uit de KiCad-layout</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Print en verbindingen</t>
         </is>
       </c>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" s="4" t="n"/>
-      <c r="H22" s="4" t="n"/>
-      <c r="I22" s="4" t="n"/>
-      <c r="J22" s="4" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Print en verbindingen</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>Level shifter 3,3 V &lt;-&gt; 5 V</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>8-kanaals bidirectionele Logic Level Converter - TXB0108</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="8" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="F23" s="8" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="G23" s="11" t="inlineStr">
-        <is>
-          <t>kiwi</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>Kiwi Electronics</t>
-        </is>
-      </c>
-      <c r="I23" s="10" t="inlineStr">
-        <is>
-          <t>https://www.kiwi-electronics.com/nl/8-channel-bi-directional-logic-level-converter-txb0108-836</t>
-        </is>
-      </c>
-      <c r="J23" s="6" t="inlineStr">
-        <is>
-          <t>Past bij de gekozen TXB-serie; antratek-alternatief BSS138-converter EUR 4,78</t>
-        </is>
-      </c>
+      <c r="B23" s="4" t="n"/>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="4" t="n"/>
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="n"/>
+      <c r="G23" s="4" t="n"/>
+      <c r="H23" s="4" t="n"/>
+      <c r="I23" s="4" t="n"/>
+      <c r="J23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -1388,37 +1413,41 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Schroefklem 4-pins 3,5 mm</t>
+          <t>Level shifter 3,3 V &lt;-&gt; 5 V</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>KF128/KF301</t>
+          <t>8-kanaals bidirectionele Logic Level Converter - TXB0108</t>
         </is>
       </c>
       <c r="D24" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>0.55</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="G24" s="14" t="inlineStr">
-        <is>
-          <t>schatting</t>
+        <v>8.699999999999999</v>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>kiwi</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>componentenwinkel</t>
-        </is>
-      </c>
-      <c r="I24" s="6" t="inlineStr"/>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="I24" s="10" t="inlineStr">
+        <is>
+          <t>https://www.kiwi-electronics.com/nl/8-channel-bi-directional-logic-level-converter-txb0108-836</t>
+        </is>
+      </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>Niet bij Kiwi (alleen 3-weg) of antratek; prijs schatting</t>
+          <t>Past bij de gekozen TXB-serie; antratek-alternatief BSS138-converter EUR 4,78</t>
         </is>
       </c>
     </row>
@@ -1430,37 +1459,41 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Sockets</t>
+          <t>Schroefklem 4-pins 3,5 mm</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Dual-wipe (ESP32) + precisie voor de rest</t>
+          <t>DEGSON DG250-3.5-04P-11-00A(H) (push-in) of KF128 (schroef)</t>
         </is>
       </c>
       <c r="D25" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>5</v>
+        <v>0.61</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="G25" s="14" t="inlineStr">
-        <is>
-          <t>schatting</t>
+        <v>0.61</v>
+      </c>
+      <c r="G25" s="18" t="inlineStr">
+        <is>
+          <t>hestore</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>componentenwinkel</t>
-        </is>
-      </c>
-      <c r="I25" s="6" t="inlineStr"/>
+          <t>HESTORE (HU, EU) / TME</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr">
+        <is>
+          <t>https://www.hestore.eu/en/prod_10044104.html</t>
+        </is>
+      </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>Niet bij Kiwi of antratek; prijs schatting (zie pcb-methodes-kosten)</t>
+          <t>Kiwi heeft alleen 3-weg; de schroefvariant KF128 is in de EU minder courant</t>
         </is>
       </c>
     </row>
@@ -1472,41 +1505,41 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Power-LED + serieweerstand</t>
+          <t>Sockets</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>3 mm LED rood (10-pack) + weerstand 330 Ohm (10-pack)</t>
+          <t>Dual-wipe (XIAO) + precisie/turned-pin (Preci-Dip) voor de rest</t>
         </is>
       </c>
       <c r="D26" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>2.16</v>
+        <v>5</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>2.16</v>
-      </c>
-      <c r="G26" s="11" t="inlineStr">
-        <is>
-          <t>kiwi</t>
+        <v>5</v>
+      </c>
+      <c r="G26" s="16" t="inlineStr">
+        <is>
+          <t>tme</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>Kiwi Electronics</t>
+          <t>TME / RS Components</t>
         </is>
       </c>
       <c r="I26" s="10" t="inlineStr">
         <is>
-          <t>https://www.kiwi-electronics.com/nl/3mm-led-diffuus-rood-10-pack-3085</t>
+          <t>https://int.rsdelivers.com/product/preci-dip/110-87-304-41-001101/preci-dip-110-254-mm-pitch-vertical-4-way-through/7020644P</t>
         </is>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>10-packs: 1 LED + 1 weerstand nodig; weerstand EUR 0,96; rest overschot</t>
+          <t>Preci-Dip turned-pin sockets via TME of RS; dual-wipe headers via Mouser/TME</t>
         </is>
       </c>
     </row>
@@ -1518,41 +1551,33 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Ontkoppelcondensatoren</t>
+          <t>Power-LED + serieweerstand</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Keramische condensator kit (15 soorten, 450 st.) - dekt 100 nF + 10 uF</t>
+          <t>3 mm LED rood (10-pack) + weerstand 330 Ohm (10-pack) - heeft de gebruiker thuis</t>
         </is>
       </c>
       <c r="D27" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E27" s="8" t="n">
-        <v>10.27</v>
-      </c>
-      <c r="F27" s="8" t="n">
-        <v>10.27</v>
-      </c>
-      <c r="G27" s="11" t="inlineStr">
-        <is>
-          <t>kiwi</t>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="5" t="n"/>
+      <c r="G27" s="13" t="inlineStr">
+        <is>
+          <t>al in bezit</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>Kiwi Electronics</t>
-        </is>
-      </c>
-      <c r="I27" s="10" t="inlineStr">
-        <is>
-          <t>https://www.kiwi-electronics.com/nl/keramische-condensator-kit-in-doos-15-soorten-450-stuks-10492</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr"/>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>Kit i.p.v. losse condensatoren</t>
+          <t>HEEFT DE GEBRUIKER THUIS (2026-10-06): 10-pack rode 3 mm LED + 10-pack 330 Ohm; niet aankopen. Referentie Kiwi: LED EUR 1,20 + weerstand EUR 0,96 = EUR 2,16</t>
         </is>
       </c>
     </row>
@@ -1564,22 +1589,22 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Bulk-elco</t>
+          <t>Ontkoppelcondensatoren</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>100 uF / 16 V op de 5 V-ingang</t>
+          <t>Keramische condensator kit (15 soorten, 450 st.) - dekt 100 nF + 10 uF</t>
         </is>
       </c>
       <c r="D28" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>0.59</v>
+        <v>10.27</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>0.59</v>
+        <v>10.27</v>
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
@@ -1593,10 +1618,14 @@
       </c>
       <c r="I28" s="10" t="inlineStr">
         <is>
-          <t>https://www.kiwi-electronics.com/nl/100uf-16v-condensator-440</t>
-        </is>
-      </c>
-      <c r="J28" s="6" t="inlineStr"/>
+          <t>https://www.kiwi-electronics.com/nl/keramische-condensator-kit-in-doos-15-soorten-450-stuks-10492</t>
+        </is>
+      </c>
+      <c r="J28" s="6" t="inlineStr">
+        <is>
+          <t>Kit i.p.v. losse condensatoren</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1606,35 +1635,39 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>I2C-pull-ups op de print</t>
+          <t>Bulk-elco</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Niet nodig; breakouts hebben ze al</t>
+          <t>100 uF / 16 V op de 5 V-ingang</t>
         </is>
       </c>
       <c r="D29" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E29" s="5" t="n"/>
-      <c r="F29" s="5" t="n"/>
-      <c r="G29" s="15" t="inlineStr">
-        <is>
-          <t>niet nodig</t>
+        <v>1</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F29" s="8" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="G29" s="11" t="inlineStr">
+        <is>
+          <t>kiwi</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I29" s="6" t="inlineStr"/>
-      <c r="J29" s="6" t="inlineStr">
-        <is>
-          <t>2 reserve-footprints</t>
-        </is>
-      </c>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="I29" s="10" t="inlineStr">
+        <is>
+          <t>https://www.kiwi-electronics.com/nl/100uf-16v-condensator-440</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -1644,89 +1677,97 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Montage</t>
+          <t>I2C-pull-ups op de print</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>M3-schroeven, moeren, standoffs, nylon spacers</t>
+          <t>Niet nodig; breakouts hebben ze al</t>
         </is>
       </c>
       <c r="D30" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="F30" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="G30" s="14" t="inlineStr">
-        <is>
-          <t>schatting</t>
+        <v>2</v>
+      </c>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="15" t="inlineStr">
+        <is>
+          <t>niet nodig</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>componentenwinkel</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr"/>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>Niet bij Kiwi of antratek; prijs schatting</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="3" t="inlineStr">
+          <t>2 reserve-footprints</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Print en verbindingen</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Montage</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>M3-schroeven, moeren, afstandsbusjes, nylon spacers</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F31" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>tinytronics</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>TinyTronics (NL, EU)</t>
+        </is>
+      </c>
+      <c r="I31" s="10" t="inlineStr">
+        <is>
+          <t>https://www.tinytronics.nl/nl/gereedschap-en-montage/installatie-en-montagemateriaal/afstandsbusjes/m3-afstandsbusje-kit</t>
+        </is>
+      </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>Alternatief: Bits &amp; Parts (NL) 180-delige M3-set EUR 6,95</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Kabels en verbruik (in bezit)</t>
         </is>
       </c>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="n"/>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="4" t="n"/>
-      <c r="H31" s="4" t="n"/>
-      <c r="I31" s="4" t="n"/>
-      <c r="J31" s="4" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>Kabels en verbruik (in bezit)</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>USB-C datakabel</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>Eigen kabel</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" s="5" t="n"/>
-      <c r="F32" s="5" t="n"/>
-      <c r="G32" s="13" t="inlineStr">
-        <is>
-          <t>al in bezit</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I32" s="6" t="inlineStr"/>
-      <c r="J32" s="6" t="inlineStr"/>
+      <c r="B32" s="4" t="n"/>
+      <c r="C32" s="4" t="n"/>
+      <c r="D32" s="4" t="n"/>
+      <c r="E32" s="4" t="n"/>
+      <c r="F32" s="4" t="n"/>
+      <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="n"/>
+      <c r="I32" s="4" t="n"/>
+      <c r="J32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -1736,12 +1777,12 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Dupont-/siliconendraad</t>
+          <t>USB-C datakabel</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Heeft de gebruiker</t>
+          <t>Eigen kabel</t>
         </is>
       </c>
       <c r="D33" s="7" t="n">
@@ -1770,12 +1811,12 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>USB A-kabel LoRa-ontvanger</t>
+          <t>Dupont-/siliconendraad</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>USB-A naar USB-C voor de XIAO (heeft de gebruiker)</t>
+          <t>Heeft de gebruiker</t>
         </is>
       </c>
       <c r="D34" s="7" t="n">
@@ -1804,12 +1845,12 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Gereedschap</t>
+          <t>USB A-kabel LoRa-ontvanger</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Schuifmaat, soldeerbout, tin, flux, multimeter, USB-serieel adapter</t>
+          <t>USB-A naar USB-C voor de XIAO (heeft de gebruiker)</t>
         </is>
       </c>
       <c r="D35" s="7" t="n">
@@ -1830,59 +1871,55 @@
       <c r="I35" s="6" t="inlineStr"/>
       <c r="J35" s="6" t="inlineStr"/>
     </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="3" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Kabels en verbruik (in bezit)</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Gereedschap</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Schuifmaat, soldeerbout, tin, flux, multimeter, USB-serieel adapter</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="5" t="n"/>
+      <c r="F36" s="5" t="n"/>
+      <c r="G36" s="13" t="inlineStr">
+        <is>
+          <t>al in bezit</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr"/>
+      <c r="J36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>Mock-up (vliegtuigje)</t>
         </is>
       </c>
-      <c r="B36" s="4" t="n"/>
-      <c r="C36" s="4" t="n"/>
-      <c r="D36" s="4" t="n"/>
-      <c r="E36" s="4" t="n"/>
-      <c r="F36" s="4" t="n"/>
-      <c r="G36" s="4" t="n"/>
-      <c r="H36" s="4" t="n"/>
-      <c r="I36" s="4" t="n"/>
-      <c r="J36" s="4" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Mock-up (vliegtuigje)</t>
-        </is>
-      </c>
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>Arduino</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>Arduino Uno (heeft de gebruiker thuis)</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" s="5" t="n"/>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="13" t="inlineStr">
-        <is>
-          <t>al in bezit</t>
-        </is>
-      </c>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I37" s="6" t="inlineStr"/>
-      <c r="J37" s="6" t="inlineStr">
-        <is>
-          <t>Referentie antratek: Arduino Uno Rev3 (EUR 41,75)</t>
-        </is>
-      </c>
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="n"/>
+      <c r="D37" s="4" t="n"/>
+      <c r="E37" s="4" t="n"/>
+      <c r="F37" s="4" t="n"/>
+      <c r="G37" s="4" t="n"/>
+      <c r="H37" s="4" t="n"/>
+      <c r="I37" s="4" t="n"/>
+      <c r="J37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -1892,16 +1929,16 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Servo's</t>
+          <t>Arduino</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Bestaande voorraad (&gt; 3)</t>
+          <t>Arduino Uno (heeft de gebruiker thuis)</t>
         </is>
       </c>
       <c r="D38" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E38" s="5" t="n"/>
       <c r="F38" s="5" t="n"/>
@@ -1916,7 +1953,11 @@
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr"/>
-      <c r="J38" s="6" t="inlineStr"/>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>Referentie antratek: Arduino Uno Rev3 (EUR 41,75)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -1926,16 +1967,16 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Servo-voeding</t>
+          <t>Servo's</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Aparte buck-converter</t>
+          <t>Bestaande voorraad (&gt; 3)</t>
         </is>
       </c>
       <c r="D39" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E39" s="5" t="n"/>
       <c r="F39" s="5" t="n"/>
@@ -1960,12 +2001,12 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Romp en roeren</t>
+          <t>Servo-voeding</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Eigen 3D-print</t>
+          <t>Aparte buck-converter</t>
         </is>
       </c>
       <c r="D40" s="7" t="n">
@@ -1986,157 +2027,275 @@
       <c r="I40" s="6" t="inlineStr"/>
       <c r="J40" s="6" t="inlineStr"/>
     </row>
-    <row r="42">
-      <c r="A42" s="17" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Mock-up (vliegtuigje)</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>Romp en roeren</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Eigen 3D-print</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="5" t="n"/>
+      <c r="F41" s="5" t="n"/>
+      <c r="G41" s="13" t="inlineStr">
+        <is>
+          <t>al in bezit</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr"/>
+      <c r="J41" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="19" t="inlineStr">
         <is>
           <t>Totaal te bestellen bij Kiwi Electronics</t>
         </is>
       </c>
-      <c r="B42" s="18" t="n"/>
-      <c r="C42" s="18" t="n"/>
-      <c r="D42" s="18" t="n"/>
-      <c r="E42" s="18" t="n"/>
-      <c r="F42" s="19">
-        <f>SUMIF(G3:G40,"kiwi",F3:F40)</f>
+      <c r="B43" s="20" t="n"/>
+      <c r="C43" s="20" t="n"/>
+      <c r="D43" s="20" t="n"/>
+      <c r="E43" s="20" t="n"/>
+      <c r="F43" s="21">
+        <f>SUMIF(G3:G41,"kiwi",F3:F41)</f>
         <v/>
       </c>
-      <c r="G42" s="18" t="n"/>
-      <c r="H42" s="18" t="n"/>
-      <c r="I42" s="18" t="n"/>
-      <c r="J42" s="18" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="17" t="inlineStr">
+      <c r="G43" s="20" t="n"/>
+      <c r="H43" s="20" t="n"/>
+      <c r="I43" s="20" t="n"/>
+      <c r="J43" s="20" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="19" t="inlineStr">
         <is>
           <t>Totaal te bestellen bij antratek</t>
         </is>
       </c>
-      <c r="B43" s="18" t="n"/>
-      <c r="C43" s="18" t="n"/>
-      <c r="D43" s="18" t="n"/>
-      <c r="E43" s="18" t="n"/>
-      <c r="F43" s="19">
-        <f>SUMIF(G3:G40,"antratek",F3:F40)</f>
+      <c r="B44" s="20" t="n"/>
+      <c r="C44" s="20" t="n"/>
+      <c r="D44" s="20" t="n"/>
+      <c r="E44" s="20" t="n"/>
+      <c r="F44" s="21">
+        <f>SUMIF(G3:G41,"antratek",F3:F41)</f>
         <v/>
       </c>
-      <c r="G43" s="18" t="n"/>
-      <c r="H43" s="18" t="n"/>
-      <c r="I43" s="18" t="n"/>
-      <c r="J43" s="18" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="17" t="inlineStr">
-        <is>
-          <t>Subtotaal onderdelen (Kiwi + antratek)</t>
-        </is>
-      </c>
-      <c r="B44" s="18" t="n"/>
-      <c r="C44" s="18" t="n"/>
-      <c r="D44" s="18" t="n"/>
-      <c r="E44" s="18" t="n"/>
-      <c r="F44" s="19">
-        <f>F42+F43</f>
+      <c r="G44" s="20" t="n"/>
+      <c r="H44" s="20" t="n"/>
+      <c r="I44" s="20" t="n"/>
+      <c r="J44" s="20" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="19" t="inlineStr">
+        <is>
+          <t>Totaal te bestellen bij Eckstein (DE, EU)</t>
+        </is>
+      </c>
+      <c r="B45" s="20" t="n"/>
+      <c r="C45" s="20" t="n"/>
+      <c r="D45" s="20" t="n"/>
+      <c r="E45" s="20" t="n"/>
+      <c r="F45" s="21">
+        <f>SUMIF(G3:G41,"eckstein",F3:F41)</f>
         <v/>
       </c>
-      <c r="G44" s="18" t="n"/>
-      <c r="H44" s="18" t="n"/>
-      <c r="I44" s="18" t="n"/>
-      <c r="J44" s="18" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="17" t="inlineStr">
+      <c r="G45" s="20" t="n"/>
+      <c r="H45" s="20" t="n"/>
+      <c r="I45" s="20" t="n"/>
+      <c r="J45" s="20" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="19" t="inlineStr">
+        <is>
+          <t>Totaal te bestellen bij TME (EU)</t>
+        </is>
+      </c>
+      <c r="B46" s="20" t="n"/>
+      <c r="C46" s="20" t="n"/>
+      <c r="D46" s="20" t="n"/>
+      <c r="E46" s="20" t="n"/>
+      <c r="F46" s="21">
+        <f>SUMIF(G3:G41,"tme",F3:F41)</f>
+        <v/>
+      </c>
+      <c r="G46" s="20" t="n"/>
+      <c r="H46" s="20" t="n"/>
+      <c r="I46" s="20" t="n"/>
+      <c r="J46" s="20" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="19" t="inlineStr">
+        <is>
+          <t>Totaal te bestellen bij Mouser/DigiKey (EU)</t>
+        </is>
+      </c>
+      <c r="B47" s="20" t="n"/>
+      <c r="C47" s="20" t="n"/>
+      <c r="D47" s="20" t="n"/>
+      <c r="E47" s="20" t="n"/>
+      <c r="F47" s="21">
+        <f>SUMIF(G3:G41,"mouser",F3:F41)</f>
+        <v/>
+      </c>
+      <c r="G47" s="20" t="n"/>
+      <c r="H47" s="20" t="n"/>
+      <c r="I47" s="20" t="n"/>
+      <c r="J47" s="20" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="19" t="inlineStr">
+        <is>
+          <t>Totaal te bestellen bij HESTORE (EU)</t>
+        </is>
+      </c>
+      <c r="B48" s="20" t="n"/>
+      <c r="C48" s="20" t="n"/>
+      <c r="D48" s="20" t="n"/>
+      <c r="E48" s="20" t="n"/>
+      <c r="F48" s="21">
+        <f>SUMIF(G3:G41,"hestore",F3:F41)</f>
+        <v/>
+      </c>
+      <c r="G48" s="20" t="n"/>
+      <c r="H48" s="20" t="n"/>
+      <c r="I48" s="20" t="n"/>
+      <c r="J48" s="20" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="19" t="inlineStr">
+        <is>
+          <t>Totaal te bestellen bij TinyTronics (NL)</t>
+        </is>
+      </c>
+      <c r="B49" s="20" t="n"/>
+      <c r="C49" s="20" t="n"/>
+      <c r="D49" s="20" t="n"/>
+      <c r="E49" s="20" t="n"/>
+      <c r="F49" s="21">
+        <f>SUMIF(G3:G41,"tinytronics",F3:F41)</f>
+        <v/>
+      </c>
+      <c r="G49" s="20" t="n"/>
+      <c r="H49" s="20" t="n"/>
+      <c r="I49" s="20" t="n"/>
+      <c r="J49" s="20" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="19" t="inlineStr">
+        <is>
+          <t>TOTAAL onderdelen - alle winkels (excl. AISLER-print)</t>
+        </is>
+      </c>
+      <c r="B50" s="20" t="n"/>
+      <c r="C50" s="20" t="n"/>
+      <c r="D50" s="20" t="n"/>
+      <c r="E50" s="20" t="n"/>
+      <c r="F50" s="21">
+        <f>F43+F44+F45+F46+F47+F48+F49</f>
+        <v/>
+      </c>
+      <c r="G50" s="20" t="n"/>
+      <c r="H50" s="20" t="n"/>
+      <c r="I50" s="20" t="n"/>
+      <c r="J50" s="20" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="19" t="inlineStr">
         <is>
           <t>Totaal draagprint bij AISLER (3 stuks)</t>
         </is>
       </c>
-      <c r="B45" s="18" t="n"/>
-      <c r="C45" s="18" t="n"/>
-      <c r="D45" s="18" t="n"/>
-      <c r="E45" s="18" t="n"/>
-      <c r="F45" s="19">
-        <f>SUMIF(G3:G40,"aisler",F3:F40)</f>
+      <c r="B51" s="20" t="n"/>
+      <c r="C51" s="20" t="n"/>
+      <c r="D51" s="20" t="n"/>
+      <c r="E51" s="20" t="n"/>
+      <c r="F51" s="21">
+        <f>SUMIF(G3:G41,"aisler",F3:F41)</f>
         <v/>
       </c>
-      <c r="G45" s="18" t="n"/>
-      <c r="H45" s="18" t="n"/>
-      <c r="I45" s="18" t="n"/>
-      <c r="J45" s="18" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="17" t="inlineStr">
-        <is>
-          <t>Totaal PCB-onderdelen (schatting, apart bestellen)</t>
-        </is>
-      </c>
-      <c r="B46" s="18" t="n"/>
-      <c r="C46" s="18" t="n"/>
-      <c r="D46" s="18" t="n"/>
-      <c r="E46" s="18" t="n"/>
-      <c r="F46" s="19">
-        <f>SUMIF(G3:G40,"schatting",F3:F40)</f>
+      <c r="G51" s="20" t="n"/>
+      <c r="H51" s="20" t="n"/>
+      <c r="I51" s="20" t="n"/>
+      <c r="J51" s="20" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="19" t="inlineStr">
+        <is>
+          <t>Totaal alles (onderdelen + AISLER-print)</t>
+        </is>
+      </c>
+      <c r="B52" s="20" t="n"/>
+      <c r="C52" s="20" t="n"/>
+      <c r="D52" s="20" t="n"/>
+      <c r="E52" s="20" t="n"/>
+      <c r="F52" s="21">
+        <f>F50+F51</f>
         <v/>
       </c>
-      <c r="G46" s="18" t="n"/>
-      <c r="H46" s="18" t="n"/>
-      <c r="I46" s="18" t="n"/>
-      <c r="J46" s="18" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="17" t="inlineStr">
-        <is>
-          <t>Totaal alles (incl. print + PCB-onderdelen)</t>
-        </is>
-      </c>
-      <c r="B47" s="18" t="n"/>
-      <c r="C47" s="18" t="n"/>
-      <c r="D47" s="18" t="n"/>
-      <c r="E47" s="18" t="n"/>
-      <c r="F47" s="19">
-        <f>F44+F45+F46</f>
-        <v/>
-      </c>
-      <c r="G47" s="18" t="n"/>
-      <c r="H47" s="18" t="n"/>
-      <c r="I47" s="18" t="n"/>
-      <c r="J47" s="18" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="20" t="inlineStr">
-        <is>
-          <t>Let op: prijzen onder voorbehoud (Kiwi Electronics + antratek + AISLER, 2026-10-06). De PCB-onderdelen op status 'schatting' zijn benaderd (o.a. sockets, discrete voeding, LDO, schroefklem, M3-montage). Het 'geen link'-onderdeel (RTK-module LC29H) is niet in de totalen opgenomen. Details: GEBRUIKER/data/bestelschema-pcb.md.</t>
+      <c r="G52" s="20" t="n"/>
+      <c r="H52" s="20" t="n"/>
+      <c r="I52" s="20" t="n"/>
+      <c r="J52" s="20" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="22" t="inlineStr">
+        <is>
+          <t>Let op: prijzen onder voorbehoud (2026-10-06). Alle voorheen 'geen link'- en 'schatting'-onderdelen zijn nu gevonden bij EU-winkels: TME (LDO, TVS, sockets), Mouser/DigiKey (PTC), HESTORE (schroefklem), TinyTronics (M3-montage) en Eckstein (LC29H(DA)-breakout, gekozen 2026-10-06). De aparte GNSS-antenne vervalt (meegeleverd met de HAT). Bestelbaarheid gecontroleerd op 2026-10-06: alles is bestelbaar; lage voorraad bij Kiwi (BMP581 4 st., condensatorkit 2 st.). De LED + 330 Ohm-weerstand (10-packs) heeft de gebruiker thuis en is dus niet meer te bestellen. Details: GEBRUIKER/data/bestelbaarheid.md en GEBRUIKER/data/bestelschema-pcb.md.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J40"/>
-  <mergeCells count="15">
+  <autoFilter ref="A2:J41"/>
+  <mergeCells count="19">
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="A23:J23"/>
+    <mergeCell ref="A32:J32"/>
+    <mergeCell ref="A48:E48"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="A45:E45"/>
+    <mergeCell ref="A13:J13"/>
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A46:E46"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="A36:J36"/>
-    <mergeCell ref="A31:J31"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A37:J37"/>
     <mergeCell ref="A43:E43"/>
-    <mergeCell ref="A22:J22"/>
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A52:E52"/>
     <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A47:E47"/>
-    <mergeCell ref="A45:E45"/>
-    <mergeCell ref="A46:E46"/>
-    <mergeCell ref="A20:J20"/>
+    <mergeCell ref="A21:J21"/>
     <mergeCell ref="A44:E44"/>
-    <mergeCell ref="A13:J13"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2148,7 +2307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2156,19 +2315,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="B1" s="21" t="inlineStr">
+      <c r="B1" s="23" t="inlineStr">
         <is>
           <t>Betekenis</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>kiwi</t>
         </is>
@@ -2180,7 +2339,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>antratek</t>
         </is>
@@ -2192,60 +2351,132 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>eckstein</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Eckstein (Duitsland, EU): Waveshare LC29H(DA)-breakout (gekozen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>tme</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TME (Polen, EU): LDO, TVS, schroefklem, precisie-sockets</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>mouser</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mouser.be / DigiKey met EU-magazijn: PTC, exacte onderdelen</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>niet nodig</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Bewust niet voorzien (bv. P-MOSFET-ompoolbeveiliging, beslissing 2026-10-06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="30" t="inlineStr">
+        <is>
+          <t>hestore</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HESTORE (Hongarije, EU): schroefklem DEGSON</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>tinytronics</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TinyTronics (Nederland, EU): M3-montagesets</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>aisler</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Gefabriceerd bij AISLER (EU); print zelf, geen componenten</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>schatting</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Prijs is een schatting; apart te bestellen bij een componentenwinkel</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="26" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>al in bezit</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Heeft de gebruiker al; niet aankopen</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="27" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="33" t="inlineStr">
         <is>
           <t>geen link</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Niet gevonden bij Kiwi of antratek; nog geen prijs</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="28" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>niet nodig</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Bewust niet voorzien</t>
         </is>
@@ -2272,14 +2503,14 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" s="34" t="inlineStr">
         <is>
           <t>Bestelschema draagprint bij AISLER - schatting (2026-10-06)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="inlineStr">
+      <c r="A2" s="35" t="inlineStr">
         <is>
           <t>AISLER-productie - 2-laags 1,6 mm HASL Budget</t>
         </is>
@@ -2296,22 +2527,22 @@
       <c r="D3" s="6" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="31" t="inlineStr">
+      <c r="A4" s="36" t="inlineStr">
         <is>
           <t>Oppervlak</t>
         </is>
       </c>
-      <c r="B4" s="31" t="inlineStr">
+      <c r="B4" s="36" t="inlineStr">
         <is>
           <t>3 stuks incl. btw</t>
         </is>
       </c>
-      <c r="C4" s="31" t="inlineStr">
+      <c r="C4" s="36" t="inlineStr">
         <is>
           <t>6 stuks incl. btw</t>
         </is>
       </c>
-      <c r="D4" s="31" t="n"/>
+      <c r="D4" s="36" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -2370,34 +2601,34 @@
       <c r="D8" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="30" t="inlineStr">
-        <is>
-          <t>Onderdelen op de print</t>
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>Onderdelen op de print (gevonden bij EU-winkels, 2026-10-06)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="36" t="inlineStr">
         <is>
           <t>Onderdeel</t>
         </is>
       </c>
-      <c r="B11" s="31" t="inlineStr">
+      <c r="B11" s="36" t="inlineStr">
         <is>
           <t>Prijs (EUR)</t>
         </is>
       </c>
-      <c r="C11" s="31" t="inlineStr">
+      <c r="C11" s="36" t="inlineStr">
         <is>
           <t>Leverancier</t>
         </is>
       </c>
-      <c r="D11" s="31" t="n"/>
+      <c r="D11" s="36" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Sockets (dual-wipe + precisie)</t>
+          <t>Sockets: dual-wipe + Preci-Dip turned-pin</t>
         </is>
       </c>
       <c r="B12" s="8" t="n">
@@ -2405,7 +2636,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>componentenwinkel (schatting)</t>
+          <t>TME / RS Components</t>
         </is>
       </c>
       <c r="D12" s="6" t="n"/>
@@ -2413,15 +2644,15 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Voedingsbescherming (2 A PTC + DMG2301L + SMBJ10A)</t>
+          <t>PTC Littelfuse 1812L200/16 + TVS SMBJ10A-TR (zonder P-MOSFET)</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>componentenwinkel (schatting)</t>
+          <t>Mouser.be / DigiKey (EU)</t>
         </is>
       </c>
       <c r="D13" s="6" t="n"/>
@@ -2429,15 +2660,15 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>LDO AP2112K-3.3</t>
+          <t>LDO AP2112K-3.3TRG1</t>
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>0.35</v>
+        <v>0.27</v>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>componentenwinkel (schatting)</t>
+          <t>TME (EU)</t>
         </is>
       </c>
       <c r="D14" s="6" t="n"/>
@@ -2445,15 +2676,15 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Schroefklem 4-pins 3,5 mm (KF128/KF301)</t>
+          <t>Schroefklem 4-pins 3,5 mm DEGSON DG250-3.5-04P</t>
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>0.55</v>
+        <v>0.61</v>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>componentenwinkel (schatting)</t>
+          <t>HESTORE / TME (EU)</t>
         </is>
       </c>
       <c r="D15" s="6" t="n"/>
@@ -2461,34 +2692,34 @@
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>M3-schroeven, moeren, standoffs, spacers</t>
+          <t>M3-schroeven, moeren, afstandsbusjes, spacers</t>
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>componentenwinkel (schatting)</t>
+          <t>TinyTronics (NL, EU)</t>
         </is>
       </c>
       <c r="D16" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="31" t="inlineStr">
+      <c r="A17" s="36" t="inlineStr">
         <is>
           <t>Subtotaal apart te bestellen</t>
         </is>
       </c>
-      <c r="B17" s="32" t="n">
-        <v>10.85</v>
-      </c>
-      <c r="C17" s="31" t="inlineStr">
-        <is>
-          <t>schatting</t>
-        </is>
-      </c>
-      <c r="D17" s="31" t="n"/>
+      <c r="B17" s="37" t="n">
+        <v>14.88</v>
+      </c>
+      <c r="C17" s="36" t="inlineStr">
+        <is>
+          <t>EU-winkels</t>
+        </is>
+      </c>
+      <c r="D17" s="36" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -2509,15 +2740,15 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>LED + serieweerstand (per bord gebruikt)</t>
+          <t>Power-LED + serieweerstand (10-packs thuis in bezit)</t>
         </is>
       </c>
       <c r="B19" s="8" t="n">
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Kiwi Electronics</t>
+          <t>Heeft de gebruiker</t>
         </is>
       </c>
       <c r="D19" s="6" t="n"/>
@@ -2555,39 +2786,39 @@
       <c r="D21" s="6" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="31" t="inlineStr">
+      <c r="A22" s="36" t="inlineStr">
         <is>
           <t>Subtotaal al in hoofd-bestellijst</t>
         </is>
       </c>
-      <c r="B22" s="32" t="n">
-        <v>10.01</v>
-      </c>
-      <c r="C22" s="31" t="inlineStr">
+      <c r="B22" s="37" t="n">
+        <v>9.789999999999999</v>
+      </c>
+      <c r="C22" s="36" t="inlineStr">
         <is>
           <t>Kiwi Electronics</t>
         </is>
       </c>
-      <c r="D22" s="31" t="n"/>
+      <c r="D22" s="36" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="31" t="inlineStr">
+      <c r="A23" s="36" t="inlineStr">
         <is>
           <t>Totaal onderdelen op de print (met TXB0108)</t>
         </is>
       </c>
-      <c r="B23" s="32" t="n">
-        <v>20.86</v>
-      </c>
-      <c r="C23" s="31" t="inlineStr">
-        <is>
-          <t>met TXB0104-IC direct: ca. 13,96</t>
-        </is>
-      </c>
-      <c r="D23" s="31" t="n"/>
+      <c r="B23" s="37" t="n">
+        <v>24.67</v>
+      </c>
+      <c r="C23" s="36" t="inlineStr">
+        <is>
+          <t>met TXB0104-IC direct: ca. 17,77</t>
+        </is>
+      </c>
+      <c r="D23" s="36" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="30" t="inlineStr">
+      <c r="A25" s="35" t="inlineStr">
         <is>
           <t>Totalen (3 borden, incl. btw)</t>
         </is>
@@ -2612,22 +2843,22 @@
         </is>
       </c>
       <c r="B27" s="8" t="n">
-        <v>20.86</v>
+        <v>24.67</v>
       </c>
       <c r="C27" s="6" t="n"/>
       <c r="D27" s="6" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="31" t="inlineStr">
+      <c r="A28" s="36" t="inlineStr">
         <is>
           <t>Totaal</t>
         </is>
       </c>
-      <c r="B28" s="32" t="n">
-        <v>53.62</v>
-      </c>
-      <c r="C28" s="31" t="n"/>
-      <c r="D28" s="31" t="n"/>
+      <c r="B28" s="37" t="n">
+        <v>57.43</v>
+      </c>
+      <c r="C28" s="36" t="n"/>
+      <c r="D28" s="36" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -2636,25 +2867,25 @@
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>10.01</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="C29" s="6" t="n"/>
       <c r="D29" s="6" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="31" t="inlineStr">
+      <c r="A30" s="36" t="inlineStr">
         <is>
           <t>Werkelijk nieuw te bestellen</t>
         </is>
       </c>
-      <c r="B30" s="32" t="n">
-        <v>43.61</v>
-      </c>
-      <c r="C30" s="31" t="n"/>
-      <c r="D30" s="31" t="n"/>
+      <c r="B30" s="37" t="n">
+        <v>47.64</v>
+      </c>
+      <c r="C30" s="36" t="n"/>
+      <c r="D30" s="36" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="30" t="inlineStr">
+      <c r="A32" s="35" t="inlineStr">
         <is>
           <t>Bestelvolgorde</t>
         </is>
@@ -2693,7 +2924,7 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>4. Tegelijk de 'schatting'-onderdelen bestellen (sockets, voeding, LDO, klem, montage)</t>
+          <t>4. Tegelijk de printonderdelen bij EU-winkels bestellen (TME, Mouser, HESTORE, TinyTronics)</t>
         </is>
       </c>
       <c r="B36" s="6" t="n"/>
@@ -2703,7 +2934,7 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>5. Kiwi/antratek-bestelling: level shifter, LED, condensatoren, bulk-elco</t>
+          <t>5. Kiwi/antratek-bestelling: level shifter, condensatoren, bulk-elco (LED + 330 Ohm heeft de gebruiker thuis)</t>
         </is>
       </c>
       <c r="B37" s="6" t="n"/>
@@ -2730,4 +2961,546 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="34" t="inlineStr">
+        <is>
+          <t>Bestelbaarheid - gecontroleerd op 2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="23" t="inlineStr">
+        <is>
+          <t>Winkel</t>
+        </is>
+      </c>
+      <c r="B2" s="23" t="inlineStr">
+        <is>
+          <t>Artikel</t>
+        </is>
+      </c>
+      <c r="C2" s="23" t="inlineStr">
+        <is>
+          <t>Voorraad</t>
+        </is>
+      </c>
+      <c r="D2" s="23" t="inlineStr">
+        <is>
+          <t>Opmerking</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Adafruit BNO085 9-DoF IMU</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>11 st.</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>prijs bevestigd</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Adafruit BMP581 barometer</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>4 st.</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>KNAPPE voorraad</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>TXB0108 level converter</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>17 st.</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>3 mm LED rood (10-pack)</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>193 st.</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>HEEFT DE GEBRUIKER THUIS - niet bestellen</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Weerstand 330 Ohm (10 st.)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>115 st.</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>HEEFT DE GEBRUIKER THUIS - niet bestellen</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Keramische condensator kit</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>2 st.</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>KNAPPE voorraad</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>100 uF / 16 V elco</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>72 st.</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>antratek.be</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>XIAO ESP32S3 + Wio-SX1262 kit</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>op voorraad</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>2x nodig</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>antratek.be</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>SMA -&gt; U.FL pigtail 150 mm</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>op voorraad</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>TME (EU)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>AP2112K-3.3TRG1 (LDO)</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>8 198</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>prijs uit snippet (TME 403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>TME (EU)</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>SMBJ10A-TR (TVS)</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>1 820</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>prijs uit snippet</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>TME (EU)</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>AO3401A (P-MOSFET)</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>22 840</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>NIET GEBRUIKT - P-MOSFET vervalt (2026-10-06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Mouser/DigiKey</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>DMG2301L-7 (P-MOSFET)</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>losse aantallen</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>NIET GEBRUIKT - P-MOSFET vervalt (2026-10-06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Mouser/DigiKey</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>1812L200/16DR (PTC 2 A 16 V)</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>14 555 / 9 900</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>TME (EU)</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Preci-Dip socket 2,54 mm</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>MOQ 380 (business)</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>niet in kleine aantallen</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>HESTORE (EU)</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>DEGSON DG250-3.5-04P (push-in)</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>&gt; 10</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>EUR 0,52 excl.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>HESTORE (EU)</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>DEGSON 15EDGK-3.5/4P (schroef)</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>&gt; 15</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>schroefvariant</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>TinyTronics (NL)</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>M3 Afstandsbusje Kit</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>EUR 8,00 incl.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Bits &amp; Parts (NL)</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>M3 spacer-set 180-delig</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>op voorraad</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>EUR 6,95 incl.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Eckstein (DE)</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Waveshare LC29H(DA) HAT 25279 (WS25279)</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>leverbaar</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>GEKOZEN - EUR 71,39 incl.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Kamami (PL)</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Waveshare LC29H(DA) HAT 25279</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>24 u</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>~EUR 63 = goedkoopste EU</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Botland (EU)</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Waveshare LC29H(DA) HAT 25279</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>op voorraad</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>EUR 70,50</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>HESTORE (EU)</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Waveshare LC29H(DA) HAT 25279</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>&gt; 2</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>~EUR 110 incl. = duur</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>